<commit_message>
modified:   FYP 2 Checklist.xlsx
</commit_message>
<xml_diff>
--- a/FYP 2 Checklist.xlsx
+++ b/FYP 2 Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d63ed5ca29abe7a/Desktop/my file/UTP/SCHOOL WORK/UNDERGRADUATE/3RD YEAR/SEM 2/FYP 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="275" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B3A8883-9DC5-4A7D-844C-6ED4D8AE1E4D}"/>
+  <xr:revisionPtr revIDLastSave="277" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4BA4AE28-2697-4C26-BB99-C22D84DCB817}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{A67127B6-E741-4082-8256-CD80F0C0B572}"/>
   </bookViews>
@@ -1208,14 +1208,12 @@
         <v>34</v>
       </c>
       <c r="E6" s="34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" s="16">
         <v>46271</v>
       </c>
-      <c r="G6" s="16">
-        <v>46271</v>
-      </c>
+      <c r="G6" s="16"/>
       <c r="H6" s="11" t="s">
         <v>65</v>
       </c>

</xml_diff>

<commit_message>
modified:   FYP 2 Checklist.xlsx new file:   dataset/clean_dataset.py new file:   dataset/eclipse_bug_records_22-07-2022.xlsx
</commit_message>
<xml_diff>
--- a/FYP 2 Checklist.xlsx
+++ b/FYP 2 Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d63ed5ca29abe7a/Desktop/my file/UTP/SCHOOL WORK/UNDERGRADUATE/3RD YEAR/SEM 2/FYP 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="277" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4BA4AE28-2697-4C26-BB99-C22D84DCB817}"/>
+  <xr:revisionPtr revIDLastSave="296" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36EFF46F-D694-446E-845F-572F3A6E24C4}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{A67127B6-E741-4082-8256-CD80F0C0B572}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="67">
   <si>
     <t>FYP II Gantt Chart</t>
   </si>
@@ -237,7 +237,10 @@
     <t>since fyp 1</t>
   </si>
   <si>
-    <t>installed python 3.13.15 and git 2.55.0.5</t>
+    <t>installed python 3.13.15, git 2.55.0.5, setup all libraries, and purchase claude API (later can claim)</t>
+  </si>
+  <si>
+    <t>use dataset eclipse_bug_records_22-07-2022.xlsx</t>
   </si>
 </sst>
 </file>
@@ -383,27 +386,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -419,64 +407,73 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
           <xfpb:xfComplement i="0"/>
         </ext>
       </extLst>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -510,6 +507,10 @@
     </a>
   </bag>
 </FeaturePropertyBags>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -846,286 +847,286 @@
       </c>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="6"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="27"/>
+      <c r="K4" s="27"/>
+      <c r="L4" s="27"/>
+      <c r="M4" s="27"/>
+      <c r="N4" s="27"/>
+      <c r="O4" s="28"/>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="8">
+      <c r="B5" s="25"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="3">
         <v>1</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="4">
         <v>2</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="4">
         <v>3</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="4">
         <v>4</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="4">
         <v>5</v>
       </c>
-      <c r="I5" s="9">
+      <c r="I5" s="4">
         <v>6</v>
       </c>
-      <c r="J5" s="9">
+      <c r="J5" s="4">
         <v>7</v>
       </c>
-      <c r="K5" s="9">
+      <c r="K5" s="4">
         <v>8</v>
       </c>
-      <c r="L5" s="9">
+      <c r="L5" s="4">
         <v>9</v>
       </c>
-      <c r="M5" s="9">
+      <c r="M5" s="4">
         <v>10</v>
       </c>
-      <c r="N5" s="9">
+      <c r="N5" s="4">
         <v>11</v>
       </c>
-      <c r="O5" s="8">
+      <c r="O5" s="3">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B6" s="10">
+      <c r="B6" s="5">
         <v>1</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="12"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
-      <c r="J6" s="13"/>
-      <c r="K6" s="13"/>
-      <c r="L6" s="13"/>
-      <c r="M6" s="13"/>
-      <c r="N6" s="13"/>
-      <c r="O6" s="13"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="8"/>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B7" s="10">
+      <c r="B7" s="5">
         <v>2</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
-      <c r="J7" s="13"/>
-      <c r="K7" s="13"/>
-      <c r="L7" s="13"/>
-      <c r="M7" s="13"/>
-      <c r="N7" s="13"/>
-      <c r="O7" s="13"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B8" s="10">
+      <c r="B8" s="5">
         <v>3</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="13"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="13"/>
-      <c r="J8" s="13"/>
-      <c r="K8" s="13"/>
-      <c r="L8" s="13"/>
-      <c r="M8" s="13"/>
-      <c r="N8" s="13"/>
-      <c r="O8" s="13"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B9" s="10">
+      <c r="B9" s="5">
         <v>4</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="13"/>
-      <c r="J9" s="13"/>
-      <c r="K9" s="13"/>
-      <c r="L9" s="13"/>
-      <c r="M9" s="13"/>
-      <c r="N9" s="13"/>
-      <c r="O9" s="13"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8"/>
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B10" s="10">
+      <c r="B10" s="5">
         <v>5</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="12"/>
-      <c r="J10" s="13"/>
-      <c r="K10" s="13"/>
-      <c r="L10" s="13"/>
-      <c r="M10" s="13"/>
-      <c r="N10" s="13"/>
-      <c r="O10" s="13"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="8"/>
+      <c r="N10" s="8"/>
+      <c r="O10" s="8"/>
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B11" s="10">
+      <c r="B11" s="5">
         <v>6</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
-      <c r="L11" s="13"/>
-      <c r="M11" s="13"/>
-      <c r="N11" s="13"/>
-      <c r="O11" s="13"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="8"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8"/>
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B12" s="10">
+      <c r="B12" s="5">
         <v>7</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="13"/>
-      <c r="J12" s="13"/>
-      <c r="K12" s="12"/>
-      <c r="L12" s="12"/>
-      <c r="M12" s="13"/>
-      <c r="N12" s="13"/>
-      <c r="O12" s="13"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="7"/>
+      <c r="L12" s="7"/>
+      <c r="M12" s="8"/>
+      <c r="N12" s="8"/>
+      <c r="O12" s="8"/>
     </row>
     <row r="13" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B13" s="10">
+      <c r="B13" s="5">
         <v>8</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="13"/>
-      <c r="J13" s="13"/>
-      <c r="K13" s="13"/>
-      <c r="L13" s="12"/>
-      <c r="M13" s="12"/>
-      <c r="N13" s="13"/>
-      <c r="O13" s="13"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="7"/>
+      <c r="M13" s="7"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="8"/>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B14" s="10">
+      <c r="B14" s="5">
         <v>9</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13"/>
-      <c r="I14" s="13"/>
-      <c r="J14" s="13"/>
-      <c r="K14" s="13"/>
-      <c r="L14" s="13"/>
-      <c r="M14" s="12"/>
-      <c r="N14" s="12"/>
-      <c r="O14" s="13"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8"/>
+      <c r="L14" s="8"/>
+      <c r="M14" s="7"/>
+      <c r="N14" s="7"/>
+      <c r="O14" s="8"/>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B15" s="10">
+      <c r="B15" s="5">
         <v>10</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="13"/>
-      <c r="J15" s="13"/>
-      <c r="K15" s="13"/>
-      <c r="L15" s="13"/>
-      <c r="M15" s="13"/>
-      <c r="N15" s="12"/>
-      <c r="O15" s="13"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
+      <c r="M15" s="8"/>
+      <c r="N15" s="7"/>
+      <c r="O15" s="8"/>
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B16" s="10">
+      <c r="B16" s="5">
         <v>11</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="13"/>
-      <c r="J16" s="13"/>
-      <c r="K16" s="13"/>
-      <c r="L16" s="13"/>
-      <c r="M16" s="13"/>
-      <c r="N16" s="12"/>
-      <c r="O16" s="12"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="8"/>
+      <c r="N16" s="7"/>
+      <c r="O16" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1139,501 +1140,503 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0363E257-1C06-40D8-9E7D-B2DA298DD784}">
-  <dimension ref="B3:J32"/>
+  <dimension ref="B3:I32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="42.21875" style="21" customWidth="1"/>
-    <col min="4" max="4" width="35.6640625" style="21" customWidth="1"/>
-    <col min="5" max="5" width="13.88671875" customWidth="1"/>
-    <col min="6" max="6" width="14.109375" customWidth="1"/>
-    <col min="7" max="7" width="14.5546875" customWidth="1"/>
-    <col min="8" max="8" width="37.21875" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" style="1"/>
+    <col min="3" max="3" width="42.21875" style="13" customWidth="1"/>
+    <col min="4" max="4" width="35.6640625" style="16" customWidth="1"/>
+    <col min="5" max="5" width="13.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="14.109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="37.21875" style="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="12" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="G4" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="H4" s="14" t="s">
+      <c r="H4" s="17" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B5" s="17">
+      <c r="B5" s="21">
         <v>1</v>
       </c>
       <c r="C5" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="D5" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="34" t="b">
+      <c r="E5" s="14" t="b">
         <v>1</v>
       </c>
-      <c r="F5" s="16">
+      <c r="F5" s="15">
         <v>46271</v>
       </c>
-      <c r="G5" s="16">
+      <c r="G5" s="15">
         <v>46271</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="H5" s="18" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B6" s="17"/>
+    <row r="6" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B6" s="21"/>
       <c r="C6" s="20"/>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F6" s="16">
+      <c r="E6" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" s="15">
         <v>46271</v>
       </c>
-      <c r="G6" s="16"/>
-      <c r="H6" s="11" t="s">
+      <c r="G6" s="15">
+        <v>46271</v>
+      </c>
+      <c r="H6" s="18" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B7" s="17">
+    <row r="7" spans="2:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="21">
         <v>2</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="E7" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F7" s="16"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="11"/>
+      <c r="E7" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="F7" s="15">
+        <v>46272</v>
+      </c>
+      <c r="G7" s="15">
+        <v>46272</v>
+      </c>
+      <c r="H7" s="29" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="27" t="s">
+      <c r="B8" s="21"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="11"/>
+      <c r="E8" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" s="15">
+        <v>46272</v>
+      </c>
+      <c r="G8" s="15">
+        <v>46272</v>
+      </c>
+      <c r="H8" s="30"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B9" s="17">
+      <c r="B9" s="21">
         <v>3</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="E9" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F9" s="16"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="11"/>
+      <c r="E9" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="18"/>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="11" t="s">
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="E10" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="11"/>
+      <c r="E10" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="18"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B11" s="17">
+      <c r="B11" s="21">
         <v>4</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="E11" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F11" s="16"/>
-      <c r="G11" s="16"/>
-      <c r="H11" s="11"/>
+      <c r="E11" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="18"/>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="11" t="s">
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="E12" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="11"/>
+      <c r="E12" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="18"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B13" s="17">
+      <c r="B13" s="21">
         <v>5</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="E13" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F13" s="16"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="11"/>
+      <c r="E13" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="18"/>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="11" t="s">
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="E14" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F14" s="16"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="11"/>
+      <c r="E14" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="18"/>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="11" t="s">
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="E15" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F15" s="16"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="11"/>
+      <c r="E15" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="18"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B16" s="17"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="11" t="s">
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="E16" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F16" s="16"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="11"/>
-    </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="11" t="s">
+      <c r="E16" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="18"/>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F17" s="16"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="11"/>
-    </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B18" s="17">
+      <c r="E17" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="18"/>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B18" s="21">
         <v>6</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="C18" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="11" t="s">
+      <c r="D18" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="E18" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="11"/>
-    </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B19" s="17"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="11" t="s">
+      <c r="E18" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="18"/>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="E19" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="28"/>
-      <c r="J19" s="29"/>
-    </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B20" s="10">
+      <c r="E19" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="18"/>
+      <c r="I19" s="1"/>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B20" s="5">
         <v>7</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D20" s="11" t="s">
+      <c r="D20" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="E20" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="28"/>
-      <c r="J20" s="29"/>
-    </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B21" s="17">
+      <c r="E20" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="1"/>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B21" s="21">
         <v>8</v>
       </c>
-      <c r="C21" s="17" t="s">
+      <c r="C21" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="D21" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="E21" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="28"/>
-      <c r="J21" s="29"/>
-    </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B22" s="17"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="11" t="s">
+      <c r="E21" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="18"/>
+      <c r="I21" s="1"/>
+    </row>
+    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B22" s="21"/>
+      <c r="C22" s="21"/>
+      <c r="D22" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="E22" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="28"/>
-      <c r="J22" s="29"/>
-    </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B23" s="10">
+      <c r="E22" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="18"/>
+      <c r="I22" s="1"/>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B23" s="5">
         <v>9</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D23" s="11" t="s">
+      <c r="D23" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="E23" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="28"/>
-      <c r="J23" s="29"/>
-    </row>
-    <row r="24" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B24" s="10">
+      <c r="E23" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="1"/>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B24" s="5">
         <v>10</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="C24" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D24" s="23" t="s">
+      <c r="D24" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="E24" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11"/>
-      <c r="H24" s="11"/>
-      <c r="I24" s="28"/>
-      <c r="J24" s="29"/>
-    </row>
-    <row r="25" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B25" s="17">
+      <c r="E24" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="18"/>
+      <c r="I24" s="1"/>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B25" s="21">
         <v>11</v>
       </c>
-      <c r="C25" s="17" t="s">
+      <c r="C25" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="D25" s="11" t="s">
+      <c r="D25" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="E25" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="28"/>
-      <c r="J25" s="29"/>
-    </row>
-    <row r="26" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B26" s="17"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="11" t="s">
+      <c r="E25" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="18"/>
+      <c r="I25" s="1"/>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
+      <c r="D26" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="E26" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="28"/>
-      <c r="J26" s="29"/>
-    </row>
-    <row r="27" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B27" s="17"/>
-      <c r="C27" s="17"/>
-      <c r="D27" s="11" t="s">
+      <c r="E26" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="18"/>
+      <c r="I26" s="1"/>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="E27" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F27" s="11"/>
-      <c r="G27" s="11"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="28"/>
-      <c r="J27" s="29"/>
-    </row>
-    <row r="28" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B28" s="17"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="11" t="s">
+      <c r="E27" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="18"/>
+      <c r="I27" s="1"/>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
+      <c r="D28" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="E28" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F28" s="11"/>
-      <c r="G28" s="11"/>
-      <c r="H28" s="11"/>
-      <c r="I28" s="28"/>
-      <c r="J28" s="29"/>
-    </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B29" s="25">
+      <c r="E28" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="18"/>
+      <c r="I28" s="1"/>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B29" s="22">
         <v>12</v>
       </c>
-      <c r="C29" s="17" t="s">
+      <c r="C29" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="D29" s="11" t="s">
+      <c r="D29" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="E29" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F29" s="11"/>
-      <c r="G29" s="11"/>
-      <c r="H29" s="11"/>
-      <c r="I29" s="28"/>
-      <c r="J29" s="29"/>
-    </row>
-    <row r="30" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B30" s="31"/>
-      <c r="C30" s="17"/>
-      <c r="D30" s="11" t="s">
+      <c r="E29" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="18"/>
+      <c r="I29" s="1"/>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B30" s="23"/>
+      <c r="C30" s="21"/>
+      <c r="D30" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="E30" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F30" s="11"/>
-      <c r="G30" s="11"/>
-      <c r="H30" s="11"/>
-      <c r="I30" s="28"/>
-      <c r="J30" s="29"/>
-    </row>
-    <row r="31" spans="2:10" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="33">
+      <c r="E30" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F30" s="5"/>
+      <c r="G30" s="5"/>
+      <c r="H30" s="18"/>
+      <c r="I30" s="1"/>
+    </row>
+    <row r="31" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="5">
         <v>13</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C31" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D31" s="32" t="s">
+      <c r="D31" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="E31" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F31" s="11"/>
-      <c r="G31" s="11"/>
-      <c r="H31" s="11"/>
-    </row>
-    <row r="32" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B32" s="33">
+      <c r="E31" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="18"/>
+    </row>
+    <row r="32" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B32" s="5">
         <v>14</v>
       </c>
-      <c r="C32" s="30" t="s">
+      <c r="C32" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="D32" s="23" t="s">
+      <c r="D32" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="E32" s="34" t="b">
-        <v>0</v>
-      </c>
-      <c r="F32" s="11"/>
-      <c r="G32" s="11"/>
-      <c r="H32" s="11"/>
+      <c r="E32" s="14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="18"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="19">
+    <mergeCell ref="H7:H8"/>
     <mergeCell ref="C29:C30"/>
     <mergeCell ref="B29:B30"/>
     <mergeCell ref="C21:C22"/>

</xml_diff>

<commit_message>
Remove large dataset file from tracking, keep local only
</commit_message>
<xml_diff>
--- a/FYP 2 Checklist.xlsx
+++ b/FYP 2 Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d63ed5ca29abe7a/Desktop/my file/UTP/SCHOOL WORK/UNDERGRADUATE/3RD YEAR/SEM 2/FYP 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="296" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36EFF46F-D694-446E-845F-572F3A6E24C4}"/>
+  <xr:revisionPtr revIDLastSave="309" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E2758EC-C769-4200-82B9-32580A8FAF3B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{A67127B6-E741-4082-8256-CD80F0C0B572}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="68">
   <si>
     <t>FYP II Gantt Chart</t>
   </si>
@@ -241,6 +241,9 @@
   </si>
   <si>
     <t>use dataset eclipse_bug_records_22-07-2022.xlsx</t>
+  </si>
+  <si>
+    <t>claude helped it</t>
   </si>
 </sst>
 </file>
@@ -442,18 +445,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -468,12 +477,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -847,30 +850,30 @@
       </c>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B4" s="24" t="s">
+      <c r="B4" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="C4" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="27"/>
-      <c r="I4" s="27"/>
-      <c r="J4" s="27"/>
-      <c r="K4" s="27"/>
-      <c r="L4" s="27"/>
-      <c r="M4" s="27"/>
-      <c r="N4" s="27"/>
-      <c r="O4" s="28"/>
+      <c r="E4" s="29"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="29"/>
+      <c r="I4" s="29"/>
+      <c r="J4" s="29"/>
+      <c r="K4" s="29"/>
+      <c r="L4" s="29"/>
+      <c r="M4" s="29"/>
+      <c r="N4" s="29"/>
+      <c r="O4" s="30"/>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B5" s="25"/>
-      <c r="C5" s="25"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="27"/>
       <c r="D5" s="3">
         <v>1</v>
       </c>
@@ -1181,10 +1184,10 @@
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B5" s="21">
+      <c r="B5" s="22">
         <v>1</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="25" t="s">
         <v>20</v>
       </c>
       <c r="D5" s="18" t="s">
@@ -1204,8 +1207,8 @@
       </c>
     </row>
     <row r="6" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B6" s="21"/>
-      <c r="C6" s="20"/>
+      <c r="B6" s="22"/>
+      <c r="C6" s="25"/>
       <c r="D6" s="18" t="s">
         <v>34</v>
       </c>
@@ -1223,10 +1226,10 @@
       </c>
     </row>
     <row r="7" spans="2:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="21">
+      <c r="B7" s="22">
         <v>2</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="22" t="s">
         <v>21</v>
       </c>
       <c r="D7" s="19" t="s">
@@ -1241,13 +1244,13 @@
       <c r="G7" s="15">
         <v>46272</v>
       </c>
-      <c r="H7" s="29" t="s">
+      <c r="H7" s="20" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B8" s="21"/>
-      <c r="C8" s="21"/>
+      <c r="B8" s="22"/>
+      <c r="C8" s="22"/>
       <c r="D8" s="19" t="s">
         <v>36</v>
       </c>
@@ -1260,43 +1263,53 @@
       <c r="G8" s="15">
         <v>46272</v>
       </c>
-      <c r="H8" s="30"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B9" s="21">
+      <c r="B9" s="22">
         <v>3</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="C9" s="22" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="19" t="s">
         <v>37</v>
       </c>
       <c r="E9" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="18"/>
+        <v>1</v>
+      </c>
+      <c r="F9" s="15">
+        <v>46272</v>
+      </c>
+      <c r="G9" s="15">
+        <v>46272</v>
+      </c>
+      <c r="H9" s="20" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B10" s="21"/>
-      <c r="C10" s="21"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
       <c r="D10" s="19" t="s">
         <v>38</v>
       </c>
       <c r="E10" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="18"/>
+        <v>1</v>
+      </c>
+      <c r="F10" s="15">
+        <v>46272</v>
+      </c>
+      <c r="G10" s="15">
+        <v>46272</v>
+      </c>
+      <c r="H10" s="21"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B11" s="21">
+      <c r="B11" s="22">
         <v>4</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="C11" s="22" t="s">
         <v>23</v>
       </c>
       <c r="D11" s="19" t="s">
@@ -1310,8 +1323,8 @@
       <c r="H11" s="18"/>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B12" s="21"/>
-      <c r="C12" s="21"/>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22"/>
       <c r="D12" s="19" t="s">
         <v>40</v>
       </c>
@@ -1323,10 +1336,10 @@
       <c r="H12" s="18"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B13" s="21">
+      <c r="B13" s="22">
         <v>5</v>
       </c>
-      <c r="C13" s="21" t="s">
+      <c r="C13" s="22" t="s">
         <v>24</v>
       </c>
       <c r="D13" s="19" t="s">
@@ -1340,8 +1353,8 @@
       <c r="H13" s="18"/>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B14" s="21"/>
-      <c r="C14" s="21"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="22"/>
       <c r="D14" s="19" t="s">
         <v>42</v>
       </c>
@@ -1353,8 +1366,8 @@
       <c r="H14" s="18"/>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B15" s="21"/>
-      <c r="C15" s="21"/>
+      <c r="B15" s="22"/>
+      <c r="C15" s="22"/>
       <c r="D15" s="19" t="s">
         <v>43</v>
       </c>
@@ -1366,8 +1379,8 @@
       <c r="H15" s="18"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B16" s="21"/>
-      <c r="C16" s="21"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="22"/>
       <c r="D16" s="19" t="s">
         <v>44</v>
       </c>
@@ -1379,8 +1392,8 @@
       <c r="H16" s="18"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
       <c r="D17" s="19" t="s">
         <v>45</v>
       </c>
@@ -1392,10 +1405,10 @@
       <c r="H17" s="18"/>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B18" s="21">
+      <c r="B18" s="22">
         <v>6</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="22" t="s">
         <v>25</v>
       </c>
       <c r="D18" s="19" t="s">
@@ -1409,8 +1422,8 @@
       <c r="H18" s="18"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B19" s="21"/>
-      <c r="C19" s="21"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
       <c r="D19" s="19" t="s">
         <v>48</v>
       </c>
@@ -1441,10 +1454,10 @@
       <c r="I20" s="1"/>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B21" s="21">
+      <c r="B21" s="22">
         <v>8</v>
       </c>
-      <c r="C21" s="21" t="s">
+      <c r="C21" s="22" t="s">
         <v>10</v>
       </c>
       <c r="D21" s="19" t="s">
@@ -1459,8 +1472,8 @@
       <c r="I21" s="1"/>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B22" s="21"/>
-      <c r="C22" s="21"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="22"/>
       <c r="D22" s="19" t="s">
         <v>51</v>
       </c>
@@ -1509,10 +1522,10 @@
       <c r="I24" s="1"/>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B25" s="21">
+      <c r="B25" s="22">
         <v>11</v>
       </c>
-      <c r="C25" s="21" t="s">
+      <c r="C25" s="22" t="s">
         <v>28</v>
       </c>
       <c r="D25" s="19" t="s">
@@ -1527,8 +1540,8 @@
       <c r="I25" s="1"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B26" s="21"/>
-      <c r="C26" s="21"/>
+      <c r="B26" s="22"/>
+      <c r="C26" s="22"/>
       <c r="D26" s="19" t="s">
         <v>56</v>
       </c>
@@ -1541,8 +1554,8 @@
       <c r="I26" s="1"/>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B27" s="21"/>
-      <c r="C27" s="21"/>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
       <c r="D27" s="19" t="s">
         <v>57</v>
       </c>
@@ -1555,8 +1568,8 @@
       <c r="I27" s="1"/>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B28" s="21"/>
-      <c r="C28" s="21"/>
+      <c r="B28" s="22"/>
+      <c r="C28" s="22"/>
       <c r="D28" s="19" t="s">
         <v>58</v>
       </c>
@@ -1569,10 +1582,10 @@
       <c r="I28" s="1"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B29" s="22">
+      <c r="B29" s="23">
         <v>12</v>
       </c>
-      <c r="C29" s="21" t="s">
+      <c r="C29" s="22" t="s">
         <v>29</v>
       </c>
       <c r="D29" s="19" t="s">
@@ -1587,8 +1600,8 @@
       <c r="I29" s="1"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B30" s="23"/>
-      <c r="C30" s="21"/>
+      <c r="B30" s="24"/>
+      <c r="C30" s="22"/>
       <c r="D30" s="19" t="s">
         <v>60</v>
       </c>
@@ -1635,7 +1648,13 @@
       <c r="H32" s="18"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="20">
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="B9:B10"/>
     <mergeCell ref="H7:H8"/>
     <mergeCell ref="C29:C30"/>
     <mergeCell ref="B29:B30"/>
@@ -1649,12 +1668,7 @@
     <mergeCell ref="B13:B17"/>
     <mergeCell ref="C18:C19"/>
     <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="H9:H10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Phase 4: NLP preprocessing and TF-IDF feature extraction
</commit_message>
<xml_diff>
--- a/FYP 2 Checklist.xlsx
+++ b/FYP 2 Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d63ed5ca29abe7a/Desktop/my file/UTP/SCHOOL WORK/UNDERGRADUATE/3RD YEAR/SEM 2/FYP 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="309" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E2758EC-C769-4200-82B9-32580A8FAF3B}"/>
+  <xr:revisionPtr revIDLastSave="311" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9DB46EC-48CA-4AA9-9E18-1B9198A5DCF1}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{A67127B6-E741-4082-8256-CD80F0C0B572}"/>
   </bookViews>
@@ -243,7 +243,7 @@
     <t>use dataset eclipse_bug_records_22-07-2022.xlsx</t>
   </si>
   <si>
-    <t>claude helped it</t>
+    <t>Data cleaning and severity mapping, done, 478,883 rows, Critical, Medium, Low mapped</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Phase 5: XGBoost training and evaluation
</commit_message>
<xml_diff>
--- a/FYP 2 Checklist.xlsx
+++ b/FYP 2 Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d63ed5ca29abe7a/Desktop/my file/UTP/SCHOOL WORK/UNDERGRADUATE/3RD YEAR/SEM 2/FYP 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="311" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9DB46EC-48CA-4AA9-9E18-1B9198A5DCF1}"/>
+  <xr:revisionPtr revIDLastSave="324" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0381D3F-70CE-4076-9E90-A6379190BE81}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{A67127B6-E741-4082-8256-CD80F0C0B572}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="69">
   <si>
     <t>FYP II Gantt Chart</t>
   </si>
@@ -244,6 +244,9 @@
   </si>
   <si>
     <t>Data cleaning and severity mapping, done, 478,883 rows, Critical, Medium, Low mapped</t>
+  </si>
+  <si>
+    <t>478,653 rows after cleaning, 5000 TF-IDF features, both output files saved</t>
   </si>
 </sst>
 </file>
@@ -1305,7 +1308,7 @@
       </c>
       <c r="H10" s="21"/>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="22">
         <v>4</v>
       </c>
@@ -1316,11 +1319,17 @@
         <v>39</v>
       </c>
       <c r="E11" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="18"/>
+        <v>1</v>
+      </c>
+      <c r="F11" s="15">
+        <v>46272</v>
+      </c>
+      <c r="G11" s="15">
+        <v>46272</v>
+      </c>
+      <c r="H11" s="20" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B12" s="22"/>
@@ -1329,11 +1338,15 @@
         <v>40</v>
       </c>
       <c r="E12" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F12" s="15"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="18"/>
+        <v>1</v>
+      </c>
+      <c r="F12" s="15">
+        <v>46272</v>
+      </c>
+      <c r="G12" s="15">
+        <v>46272</v>
+      </c>
+      <c r="H12" s="21"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B13" s="22">
@@ -1648,7 +1661,7 @@
       <c r="H32" s="18"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="21">
     <mergeCell ref="C5:C6"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="C7:C8"/>
@@ -1669,6 +1682,7 @@
     <mergeCell ref="C18:C19"/>
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="H9:H10"/>
+    <mergeCell ref="H11:H12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Phase 5: tuned model with product/component features
</commit_message>
<xml_diff>
--- a/FYP 2 Checklist.xlsx
+++ b/FYP 2 Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d63ed5ca29abe7a/Desktop/my file/UTP/SCHOOL WORK/UNDERGRADUATE/3RD YEAR/SEM 2/FYP 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="324" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0381D3F-70CE-4076-9E90-A6379190BE81}"/>
+  <xr:revisionPtr revIDLastSave="341" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59A1805E-E224-47E0-80A0-4BD092F68CDF}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{A67127B6-E741-4082-8256-CD80F0C0B572}"/>
   </bookViews>
@@ -302,7 +302,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -388,11 +388,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -439,33 +450,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -480,6 +488,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -853,30 +867,30 @@
       </c>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="26" t="s">
+      <c r="C4" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="D4" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="29"/>
-      <c r="F4" s="29"/>
-      <c r="G4" s="29"/>
-      <c r="H4" s="29"/>
-      <c r="I4" s="29"/>
-      <c r="J4" s="29"/>
-      <c r="K4" s="29"/>
-      <c r="L4" s="29"/>
-      <c r="M4" s="29"/>
-      <c r="N4" s="29"/>
-      <c r="O4" s="30"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="28"/>
+      <c r="I4" s="28"/>
+      <c r="J4" s="28"/>
+      <c r="K4" s="28"/>
+      <c r="L4" s="28"/>
+      <c r="M4" s="28"/>
+      <c r="N4" s="28"/>
+      <c r="O4" s="29"/>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B5" s="27"/>
-      <c r="C5" s="27"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="26"/>
       <c r="D5" s="3">
         <v>1</v>
       </c>
@@ -1170,7 +1184,7 @@
       <c r="C4" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="31" t="s">
         <v>32</v>
       </c>
       <c r="E4" s="9" t="s">
@@ -1182,18 +1196,18 @@
       <c r="G4" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="H4" s="17" t="s">
+      <c r="H4" s="31" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B5" s="22">
+      <c r="B5" s="20">
         <v>1</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="17" t="s">
         <v>33</v>
       </c>
       <c r="E5" s="14" t="b">
@@ -1205,14 +1219,14 @@
       <c r="G5" s="15">
         <v>46271</v>
       </c>
-      <c r="H5" s="18" t="s">
+      <c r="H5" s="17" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B6" s="22"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="18" t="s">
+      <c r="B6" s="20"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="17" t="s">
         <v>34</v>
       </c>
       <c r="E6" s="14" t="b">
@@ -1224,18 +1238,18 @@
       <c r="G6" s="15">
         <v>46271</v>
       </c>
-      <c r="H6" s="18" t="s">
+      <c r="H6" s="17" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="22">
+      <c r="B7" s="20">
         <v>2</v>
       </c>
-      <c r="C7" s="22" t="s">
+      <c r="C7" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="18" t="s">
         <v>35</v>
       </c>
       <c r="E7" s="14" t="b">
@@ -1247,14 +1261,14 @@
       <c r="G7" s="15">
         <v>46272</v>
       </c>
-      <c r="H7" s="20" t="s">
+      <c r="H7" s="21" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B8" s="22"/>
-      <c r="C8" s="22"/>
-      <c r="D8" s="19" t="s">
+      <c r="B8" s="20"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="18" t="s">
         <v>36</v>
       </c>
       <c r="E8" s="14" t="b">
@@ -1266,16 +1280,16 @@
       <c r="G8" s="15">
         <v>46272</v>
       </c>
-      <c r="H8" s="21"/>
+      <c r="H8" s="22"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B9" s="22">
+      <c r="B9" s="20">
         <v>3</v>
       </c>
-      <c r="C9" s="22" t="s">
+      <c r="C9" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="18" t="s">
         <v>37</v>
       </c>
       <c r="E9" s="14" t="b">
@@ -1287,14 +1301,14 @@
       <c r="G9" s="15">
         <v>46272</v>
       </c>
-      <c r="H9" s="20" t="s">
+      <c r="H9" s="21" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="19" t="s">
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="18" t="s">
         <v>38</v>
       </c>
       <c r="E10" s="14" t="b">
@@ -1306,16 +1320,16 @@
       <c r="G10" s="15">
         <v>46272</v>
       </c>
-      <c r="H10" s="21"/>
+      <c r="H10" s="22"/>
     </row>
     <row r="11" spans="2:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="22">
+      <c r="B11" s="20">
         <v>4</v>
       </c>
-      <c r="C11" s="22" t="s">
+      <c r="C11" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="18" t="s">
         <v>39</v>
       </c>
       <c r="E11" s="14" t="b">
@@ -1327,14 +1341,14 @@
       <c r="G11" s="15">
         <v>46272</v>
       </c>
-      <c r="H11" s="20" t="s">
+      <c r="H11" s="21" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B12" s="22"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="19" t="s">
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="18" t="s">
         <v>40</v>
       </c>
       <c r="E12" s="14" t="b">
@@ -1346,68 +1360,84 @@
       <c r="G12" s="15">
         <v>46272</v>
       </c>
-      <c r="H12" s="21"/>
+      <c r="H12" s="22"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B13" s="22">
+      <c r="B13" s="20">
         <v>5</v>
       </c>
-      <c r="C13" s="22" t="s">
+      <c r="C13" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="D13" s="19" t="s">
+      <c r="D13" s="18" t="s">
         <v>41</v>
       </c>
       <c r="E13" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="18"/>
+        <v>1</v>
+      </c>
+      <c r="F13" s="15">
+        <v>46272</v>
+      </c>
+      <c r="G13" s="15">
+        <v>46272</v>
+      </c>
+      <c r="H13" s="21"/>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B14" s="22"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="19" t="s">
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="18" t="s">
         <v>42</v>
       </c>
       <c r="E14" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="18"/>
+        <v>1</v>
+      </c>
+      <c r="F14" s="15">
+        <v>46272</v>
+      </c>
+      <c r="G14" s="15">
+        <v>46272</v>
+      </c>
+      <c r="H14" s="30"/>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B15" s="22"/>
-      <c r="C15" s="22"/>
-      <c r="D15" s="19" t="s">
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="18" t="s">
         <v>43</v>
       </c>
       <c r="E15" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="18"/>
+        <v>1</v>
+      </c>
+      <c r="F15" s="15">
+        <v>46272</v>
+      </c>
+      <c r="G15" s="15">
+        <v>46272</v>
+      </c>
+      <c r="H15" s="30"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B16" s="22"/>
-      <c r="C16" s="22"/>
-      <c r="D16" s="19" t="s">
+      <c r="B16" s="20"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="18" t="s">
         <v>44</v>
       </c>
       <c r="E16" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="18"/>
+        <v>1</v>
+      </c>
+      <c r="F16" s="15">
+        <v>46272</v>
+      </c>
+      <c r="G16" s="15">
+        <v>46272</v>
+      </c>
+      <c r="H16" s="30"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B17" s="22"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="19" t="s">
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="18" t="s">
         <v>45</v>
       </c>
       <c r="E17" s="14" t="b">
@@ -1415,16 +1445,16 @@
       </c>
       <c r="F17" s="15"/>
       <c r="G17" s="15"/>
-      <c r="H17" s="18"/>
+      <c r="H17" s="22"/>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B18" s="22">
+      <c r="B18" s="20">
         <v>6</v>
       </c>
-      <c r="C18" s="22" t="s">
+      <c r="C18" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="19" t="s">
+      <c r="D18" s="18" t="s">
         <v>47</v>
       </c>
       <c r="E18" s="14" t="b">
@@ -1432,12 +1462,12 @@
       </c>
       <c r="F18" s="15"/>
       <c r="G18" s="15"/>
-      <c r="H18" s="18"/>
+      <c r="H18" s="21"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="19" t="s">
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="18" t="s">
         <v>48</v>
       </c>
       <c r="E19" s="14" t="b">
@@ -1445,7 +1475,7 @@
       </c>
       <c r="F19" s="5"/>
       <c r="G19" s="5"/>
-      <c r="H19" s="18"/>
+      <c r="H19" s="22"/>
       <c r="I19" s="1"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.3">
@@ -1455,7 +1485,7 @@
       <c r="C20" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D20" s="19" t="s">
+      <c r="D20" s="18" t="s">
         <v>49</v>
       </c>
       <c r="E20" s="14" t="b">
@@ -1463,17 +1493,17 @@
       </c>
       <c r="F20" s="5"/>
       <c r="G20" s="5"/>
-      <c r="H20" s="18"/>
+      <c r="H20" s="17"/>
       <c r="I20" s="1"/>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B21" s="22">
+      <c r="B21" s="20">
         <v>8</v>
       </c>
-      <c r="C21" s="22" t="s">
+      <c r="C21" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="D21" s="19" t="s">
+      <c r="D21" s="18" t="s">
         <v>50</v>
       </c>
       <c r="E21" s="14" t="b">
@@ -1481,13 +1511,13 @@
       </c>
       <c r="F21" s="5"/>
       <c r="G21" s="5"/>
-      <c r="H21" s="18"/>
+      <c r="H21" s="21"/>
       <c r="I21" s="1"/>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B22" s="22"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="19" t="s">
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="18" t="s">
         <v>51</v>
       </c>
       <c r="E22" s="14" t="b">
@@ -1495,7 +1525,7 @@
       </c>
       <c r="F22" s="5"/>
       <c r="G22" s="5"/>
-      <c r="H22" s="18"/>
+      <c r="H22" s="22"/>
       <c r="I22" s="1"/>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.3">
@@ -1505,7 +1535,7 @@
       <c r="C23" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D23" s="19" t="s">
+      <c r="D23" s="18" t="s">
         <v>52</v>
       </c>
       <c r="E23" s="14" t="b">
@@ -1513,7 +1543,7 @@
       </c>
       <c r="F23" s="5"/>
       <c r="G23" s="5"/>
-      <c r="H23" s="18"/>
+      <c r="H23" s="17"/>
       <c r="I23" s="1"/>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.3">
@@ -1523,7 +1553,7 @@
       <c r="C24" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D24" s="18" t="s">
+      <c r="D24" s="17" t="s">
         <v>54</v>
       </c>
       <c r="E24" s="14" t="b">
@@ -1531,17 +1561,17 @@
       </c>
       <c r="F24" s="5"/>
       <c r="G24" s="5"/>
-      <c r="H24" s="18"/>
+      <c r="H24" s="17"/>
       <c r="I24" s="1"/>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B25" s="22">
+      <c r="B25" s="20">
         <v>11</v>
       </c>
-      <c r="C25" s="22" t="s">
+      <c r="C25" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="D25" s="19" t="s">
+      <c r="D25" s="18" t="s">
         <v>55</v>
       </c>
       <c r="E25" s="14" t="b">
@@ -1549,13 +1579,13 @@
       </c>
       <c r="F25" s="5"/>
       <c r="G25" s="5"/>
-      <c r="H25" s="18"/>
+      <c r="H25" s="21"/>
       <c r="I25" s="1"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B26" s="22"/>
-      <c r="C26" s="22"/>
-      <c r="D26" s="19" t="s">
+      <c r="B26" s="20"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="18" t="s">
         <v>56</v>
       </c>
       <c r="E26" s="14" t="b">
@@ -1563,13 +1593,13 @@
       </c>
       <c r="F26" s="5"/>
       <c r="G26" s="5"/>
-      <c r="H26" s="18"/>
+      <c r="H26" s="30"/>
       <c r="I26" s="1"/>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B27" s="22"/>
-      <c r="C27" s="22"/>
-      <c r="D27" s="19" t="s">
+      <c r="B27" s="20"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="18" t="s">
         <v>57</v>
       </c>
       <c r="E27" s="14" t="b">
@@ -1577,13 +1607,13 @@
       </c>
       <c r="F27" s="5"/>
       <c r="G27" s="5"/>
-      <c r="H27" s="18"/>
+      <c r="H27" s="30"/>
       <c r="I27" s="1"/>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B28" s="22"/>
-      <c r="C28" s="22"/>
-      <c r="D28" s="19" t="s">
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="18" t="s">
         <v>58</v>
       </c>
       <c r="E28" s="14" t="b">
@@ -1591,17 +1621,17 @@
       </c>
       <c r="F28" s="5"/>
       <c r="G28" s="5"/>
-      <c r="H28" s="18"/>
+      <c r="H28" s="22"/>
       <c r="I28" s="1"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B29" s="23">
         <v>12</v>
       </c>
-      <c r="C29" s="22" t="s">
+      <c r="C29" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="D29" s="19" t="s">
+      <c r="D29" s="18" t="s">
         <v>59</v>
       </c>
       <c r="E29" s="14" t="b">
@@ -1609,13 +1639,13 @@
       </c>
       <c r="F29" s="5"/>
       <c r="G29" s="5"/>
-      <c r="H29" s="18"/>
+      <c r="H29" s="21"/>
       <c r="I29" s="1"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B30" s="24"/>
-      <c r="C30" s="22"/>
-      <c r="D30" s="19" t="s">
+      <c r="C30" s="20"/>
+      <c r="D30" s="18" t="s">
         <v>60</v>
       </c>
       <c r="E30" s="14" t="b">
@@ -1623,7 +1653,7 @@
       </c>
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
-      <c r="H30" s="18"/>
+      <c r="H30" s="22"/>
       <c r="I30" s="1"/>
     </row>
     <row r="31" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -1633,7 +1663,7 @@
       <c r="C31" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D31" s="18" t="s">
+      <c r="D31" s="17" t="s">
         <v>61</v>
       </c>
       <c r="E31" s="14" t="b">
@@ -1641,7 +1671,7 @@
       </c>
       <c r="F31" s="5"/>
       <c r="G31" s="5"/>
-      <c r="H31" s="18"/>
+      <c r="H31" s="17"/>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B32" s="5">
@@ -1650,7 +1680,7 @@
       <c r="C32" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="D32" s="18" t="s">
+      <c r="D32" s="17" t="s">
         <v>62</v>
       </c>
       <c r="E32" s="14" t="b">
@@ -1658,16 +1688,14 @@
       </c>
       <c r="F32" s="5"/>
       <c r="G32" s="5"/>
-      <c r="H32" s="18"/>
+      <c r="H32" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="21">
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="B9:B10"/>
+  <mergeCells count="26">
+    <mergeCell ref="H18:H19"/>
+    <mergeCell ref="H21:H22"/>
+    <mergeCell ref="H25:H28"/>
+    <mergeCell ref="H29:H30"/>
     <mergeCell ref="H7:H8"/>
     <mergeCell ref="C29:C30"/>
     <mergeCell ref="B29:B30"/>
@@ -1683,6 +1711,13 @@
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="H9:H10"/>
     <mergeCell ref="H11:H12"/>
+    <mergeCell ref="H13:H17"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="B9:B10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Phase 6: Flask backend and bug submission form
</commit_message>
<xml_diff>
--- a/FYP 2 Checklist.xlsx
+++ b/FYP 2 Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d63ed5ca29abe7a/Desktop/my file/UTP/SCHOOL WORK/UNDERGRADUATE/3RD YEAR/SEM 2/FYP 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="341" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59A1805E-E224-47E0-80A0-4BD092F68CDF}"/>
+  <xr:revisionPtr revIDLastSave="345" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B16A1E4-B9BF-410E-84EB-9EA77D6F0739}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{A67127B6-E741-4082-8256-CD80F0C0B572}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="70">
   <si>
     <t>FYP II Gantt Chart</t>
   </si>
@@ -247,6 +247,9 @@
   </si>
   <si>
     <t>478,653 rows after cleaning, 5000 TF-IDF features, both output files saved</t>
+  </si>
+  <si>
+    <t>tuned model with product and component features</t>
   </si>
 </sst>
 </file>
@@ -1381,7 +1384,9 @@
       <c r="G13" s="15">
         <v>46272</v>
       </c>
-      <c r="H13" s="21"/>
+      <c r="H13" s="21" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B14" s="20"/>
@@ -1441,10 +1446,14 @@
         <v>45</v>
       </c>
       <c r="E17" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
+        <v>1</v>
+      </c>
+      <c r="F17" s="15">
+        <v>46272</v>
+      </c>
+      <c r="G17" s="15">
+        <v>46272</v>
+      </c>
       <c r="H17" s="22"/>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Phase 7: connected trained XGBoost model to Flask
</commit_message>
<xml_diff>
--- a/FYP 2 Checklist.xlsx
+++ b/FYP 2 Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d63ed5ca29abe7a/Desktop/my file/UTP/SCHOOL WORK/UNDERGRADUATE/3RD YEAR/SEM 2/FYP 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="345" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B16A1E4-B9BF-410E-84EB-9EA77D6F0739}"/>
+  <xr:revisionPtr revIDLastSave="349" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FAD79182-18B4-4639-8265-92F7871D7984}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{A67127B6-E741-4082-8256-CD80F0C0B572}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="71">
   <si>
     <t>FYP II Gantt Chart</t>
   </si>
@@ -250,6 +250,9 @@
   </si>
   <si>
     <t>tuned model with product and component features</t>
+  </si>
+  <si>
+    <t>building the first phase of web application development</t>
   </si>
 </sst>
 </file>
@@ -1467,11 +1470,17 @@
         <v>47</v>
       </c>
       <c r="E18" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="21"/>
+        <v>1</v>
+      </c>
+      <c r="F18" s="15">
+        <v>46272</v>
+      </c>
+      <c r="G18" s="15">
+        <v>46272</v>
+      </c>
+      <c r="H18" s="21" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B19" s="20"/>
@@ -1480,10 +1489,14 @@
         <v>48</v>
       </c>
       <c r="E19" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="F19" s="15">
+        <v>46272</v>
+      </c>
+      <c r="G19" s="15">
+        <v>46272</v>
+      </c>
       <c r="H19" s="22"/>
       <c r="I19" s="1"/>
     </row>

</xml_diff>

<commit_message>
Phase 9 and 10: dashboard, authetication, MySQL database
</commit_message>
<xml_diff>
--- a/FYP 2 Checklist.xlsx
+++ b/FYP 2 Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d63ed5ca29abe7a/Desktop/my file/UTP/SCHOOL WORK/UNDERGRADUATE/3RD YEAR/SEM 2/FYP 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="353" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6C0DB3EF-5350-4BCE-94A8-78680D3CCA46}"/>
+  <xr:revisionPtr revIDLastSave="367" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E22AE2E-082F-4B3A-9366-14BFBB38D1EE}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{A67127B6-E741-4082-8256-CD80F0C0B572}"/>
   </bookViews>
@@ -17,6 +17,7 @@
     <sheet name="roadmap" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="75">
   <si>
     <t>FYP II Gantt Chart</t>
   </si>
@@ -256,6 +257,15 @@
   </si>
   <si>
     <t>Real model connected, tested with Critical and Low examples, done. Connected trained XGBoost model to Flask</t>
+  </si>
+  <si>
+    <t>connected Claude API for solution recommendations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">first phase, later will update and enhance </t>
+  </si>
+  <si>
+    <t>auto filled right after the code is runnung</t>
   </si>
 </sst>
 </file>
@@ -465,6 +475,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -472,16 +485,19 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -497,12 +513,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -876,30 +886,30 @@
       </c>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B4" s="25" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="25" t="s">
+      <c r="B4" s="27" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="27" t="s">
+      <c r="D4" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="28"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="28"/>
-      <c r="I4" s="28"/>
-      <c r="J4" s="28"/>
-      <c r="K4" s="28"/>
-      <c r="L4" s="28"/>
-      <c r="M4" s="28"/>
-      <c r="N4" s="28"/>
-      <c r="O4" s="29"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
+      <c r="L4" s="30"/>
+      <c r="M4" s="30"/>
+      <c r="N4" s="30"/>
+      <c r="O4" s="31"/>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B5" s="26"/>
-      <c r="C5" s="26"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
       <c r="D5" s="3">
         <v>1</v>
       </c>
@@ -1193,7 +1203,7 @@
       <c r="C4" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="D4" s="31" t="s">
+      <c r="D4" s="19" t="s">
         <v>32</v>
       </c>
       <c r="E4" s="9" t="s">
@@ -1205,15 +1215,15 @@
       <c r="G4" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="H4" s="31" t="s">
+      <c r="H4" s="19" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B5" s="20">
-        <v>1</v>
-      </c>
-      <c r="C5" s="19" t="s">
+      <c r="B5" s="21">
+        <v>1</v>
+      </c>
+      <c r="C5" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D5" s="17" t="s">
@@ -1233,8 +1243,8 @@
       </c>
     </row>
     <row r="6" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B6" s="20"/>
-      <c r="C6" s="19"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="20"/>
       <c r="D6" s="17" t="s">
         <v>34</v>
       </c>
@@ -1252,10 +1262,10 @@
       </c>
     </row>
     <row r="7" spans="2:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="20">
+      <c r="B7" s="21">
         <v>2</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="C7" s="21" t="s">
         <v>21</v>
       </c>
       <c r="D7" s="18" t="s">
@@ -1270,13 +1280,13 @@
       <c r="G7" s="15">
         <v>46272</v>
       </c>
-      <c r="H7" s="21" t="s">
+      <c r="H7" s="24" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="21"/>
       <c r="D8" s="18" t="s">
         <v>36</v>
       </c>
@@ -1289,13 +1299,13 @@
       <c r="G8" s="15">
         <v>46272</v>
       </c>
-      <c r="H8" s="22"/>
+      <c r="H8" s="25"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B9" s="20">
+      <c r="B9" s="21">
         <v>3</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="C9" s="21" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="18" t="s">
@@ -1310,13 +1320,13 @@
       <c r="G9" s="15">
         <v>46272</v>
       </c>
-      <c r="H9" s="21" t="s">
+      <c r="H9" s="24" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
       <c r="D10" s="18" t="s">
         <v>38</v>
       </c>
@@ -1329,13 +1339,13 @@
       <c r="G10" s="15">
         <v>46272</v>
       </c>
-      <c r="H10" s="22"/>
+      <c r="H10" s="25"/>
     </row>
     <row r="11" spans="2:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="20">
+      <c r="B11" s="21">
         <v>4</v>
       </c>
-      <c r="C11" s="20" t="s">
+      <c r="C11" s="21" t="s">
         <v>23</v>
       </c>
       <c r="D11" s="18" t="s">
@@ -1350,13 +1360,13 @@
       <c r="G11" s="15">
         <v>46272</v>
       </c>
-      <c r="H11" s="21" t="s">
+      <c r="H11" s="24" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
       <c r="D12" s="18" t="s">
         <v>40</v>
       </c>
@@ -1369,13 +1379,13 @@
       <c r="G12" s="15">
         <v>46272</v>
       </c>
-      <c r="H12" s="22"/>
+      <c r="H12" s="25"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B13" s="20">
+      <c r="B13" s="21">
         <v>5</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="C13" s="21" t="s">
         <v>24</v>
       </c>
       <c r="D13" s="18" t="s">
@@ -1390,13 +1400,13 @@
       <c r="G13" s="15">
         <v>46272</v>
       </c>
-      <c r="H13" s="21" t="s">
+      <c r="H13" s="24" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
       <c r="D14" s="18" t="s">
         <v>42</v>
       </c>
@@ -1409,11 +1419,11 @@
       <c r="G14" s="15">
         <v>46272</v>
       </c>
-      <c r="H14" s="30"/>
+      <c r="H14" s="26"/>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
       <c r="D15" s="18" t="s">
         <v>43</v>
       </c>
@@ -1426,11 +1436,11 @@
       <c r="G15" s="15">
         <v>46272</v>
       </c>
-      <c r="H15" s="30"/>
+      <c r="H15" s="26"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
       <c r="D16" s="18" t="s">
         <v>44</v>
       </c>
@@ -1443,11 +1453,11 @@
       <c r="G16" s="15">
         <v>46272</v>
       </c>
-      <c r="H16" s="30"/>
+      <c r="H16" s="26"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
       <c r="D17" s="18" t="s">
         <v>45</v>
       </c>
@@ -1460,13 +1470,13 @@
       <c r="G17" s="15">
         <v>46272</v>
       </c>
-      <c r="H17" s="22"/>
+      <c r="H17" s="25"/>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B18" s="20">
+      <c r="B18" s="21">
         <v>6</v>
       </c>
-      <c r="C18" s="20" t="s">
+      <c r="C18" s="21" t="s">
         <v>25</v>
       </c>
       <c r="D18" s="18" t="s">
@@ -1481,13 +1491,13 @@
       <c r="G18" s="15">
         <v>46272</v>
       </c>
-      <c r="H18" s="21" t="s">
+      <c r="H18" s="24" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
       <c r="D19" s="18" t="s">
         <v>48</v>
       </c>
@@ -1500,7 +1510,7 @@
       <c r="G19" s="15">
         <v>46272</v>
       </c>
-      <c r="H19" s="22"/>
+      <c r="H19" s="25"/>
       <c r="I19" s="1"/>
     </row>
     <row r="20" spans="2:9" ht="43.2" x14ac:dyDescent="0.3">
@@ -1528,35 +1538,45 @@
       <c r="I20" s="1"/>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B21" s="20">
+      <c r="B21" s="21">
         <v>8</v>
       </c>
-      <c r="C21" s="20" t="s">
+      <c r="C21" s="21" t="s">
         <v>10</v>
       </c>
       <c r="D21" s="18" t="s">
         <v>50</v>
       </c>
       <c r="E21" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="21"/>
+        <v>1</v>
+      </c>
+      <c r="F21" s="15">
+        <v>46274</v>
+      </c>
+      <c r="G21" s="15">
+        <v>46274</v>
+      </c>
+      <c r="H21" s="24" t="s">
+        <v>72</v>
+      </c>
       <c r="I21" s="1"/>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="21"/>
       <c r="D22" s="18" t="s">
         <v>51</v>
       </c>
       <c r="E22" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="22"/>
+        <v>1</v>
+      </c>
+      <c r="F22" s="15">
+        <v>46274</v>
+      </c>
+      <c r="G22" s="15">
+        <v>46274</v>
+      </c>
+      <c r="H22" s="25"/>
       <c r="I22" s="1"/>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.3">
@@ -1570,11 +1590,17 @@
         <v>52</v>
       </c>
       <c r="E23" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-      <c r="H23" s="17"/>
+        <v>1</v>
+      </c>
+      <c r="F23" s="15">
+        <v>46274</v>
+      </c>
+      <c r="G23" s="15">
+        <v>46274</v>
+      </c>
+      <c r="H23" s="17" t="s">
+        <v>73</v>
+      </c>
       <c r="I23" s="1"/>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.3">
@@ -1588,18 +1614,24 @@
         <v>54</v>
       </c>
       <c r="E24" s="14" t="b">
-        <v>0</v>
-      </c>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
-      <c r="H24" s="17"/>
+        <v>1</v>
+      </c>
+      <c r="F24" s="15">
+        <v>46274</v>
+      </c>
+      <c r="G24" s="15">
+        <v>46274</v>
+      </c>
+      <c r="H24" s="17" t="s">
+        <v>74</v>
+      </c>
       <c r="I24" s="1"/>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B25" s="20">
+      <c r="B25" s="21">
         <v>11</v>
       </c>
-      <c r="C25" s="20" t="s">
+      <c r="C25" s="21" t="s">
         <v>28</v>
       </c>
       <c r="D25" s="18" t="s">
@@ -1608,58 +1640,58 @@
       <c r="E25" s="14" t="b">
         <v>0</v>
       </c>
-      <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
-      <c r="H25" s="21"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="24"/>
       <c r="I25" s="1"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
       <c r="D26" s="18" t="s">
         <v>56</v>
       </c>
       <c r="E26" s="14" t="b">
         <v>0</v>
       </c>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
-      <c r="H26" s="30"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="15"/>
+      <c r="H26" s="26"/>
       <c r="I26" s="1"/>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B27" s="20"/>
-      <c r="C27" s="20"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
       <c r="D27" s="18" t="s">
         <v>57</v>
       </c>
       <c r="E27" s="14" t="b">
         <v>0</v>
       </c>
-      <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
-      <c r="H27" s="30"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="15"/>
+      <c r="H27" s="26"/>
       <c r="I27" s="1"/>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
       <c r="D28" s="18" t="s">
         <v>58</v>
       </c>
       <c r="E28" s="14" t="b">
         <v>0</v>
       </c>
-      <c r="F28" s="5"/>
-      <c r="G28" s="5"/>
-      <c r="H28" s="22"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="25"/>
       <c r="I28" s="1"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B29" s="23">
+      <c r="B29" s="22">
         <v>12</v>
       </c>
-      <c r="C29" s="20" t="s">
+      <c r="C29" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D29" s="18" t="s">
@@ -1668,23 +1700,23 @@
       <c r="E29" s="14" t="b">
         <v>0</v>
       </c>
-      <c r="F29" s="5"/>
-      <c r="G29" s="5"/>
-      <c r="H29" s="21"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="24"/>
       <c r="I29" s="1"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B30" s="24"/>
-      <c r="C30" s="20"/>
+      <c r="B30" s="23"/>
+      <c r="C30" s="21"/>
       <c r="D30" s="18" t="s">
         <v>60</v>
       </c>
       <c r="E30" s="14" t="b">
         <v>0</v>
       </c>
-      <c r="F30" s="5"/>
-      <c r="G30" s="5"/>
-      <c r="H30" s="22"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="15"/>
+      <c r="H30" s="25"/>
       <c r="I30" s="1"/>
     </row>
     <row r="31" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -1700,8 +1732,8 @@
       <c r="E31" s="14" t="b">
         <v>0</v>
       </c>
-      <c r="F31" s="5"/>
-      <c r="G31" s="5"/>
+      <c r="F31" s="15"/>
+      <c r="G31" s="15"/>
       <c r="H31" s="17"/>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.3">
@@ -1717,8 +1749,8 @@
       <c r="E32" s="14" t="b">
         <v>0</v>
       </c>
-      <c r="F32" s="5"/>
-      <c r="G32" s="5"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="15"/>
       <c r="H32" s="17"/>
     </row>
   </sheetData>
@@ -1728,6 +1760,9 @@
     <mergeCell ref="H25:H28"/>
     <mergeCell ref="H29:H30"/>
     <mergeCell ref="H7:H8"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="H13:H17"/>
     <mergeCell ref="C29:C30"/>
     <mergeCell ref="B29:B30"/>
     <mergeCell ref="C21:C22"/>
@@ -1740,9 +1775,6 @@
     <mergeCell ref="B13:B17"/>
     <mergeCell ref="C18:C19"/>
     <mergeCell ref="B18:B19"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="H13:H17"/>
     <mergeCell ref="C5:C6"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="C7:C8"/>

</xml_diff>

<commit_message>
fix refresh page for Reports page & change sidebar ui
</commit_message>
<xml_diff>
--- a/FYP 2 Checklist.xlsx
+++ b/FYP 2 Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d63ed5ca29abe7a/Desktop/my file/UTP/SCHOOL WORK/UNDERGRADUATE/3RD YEAR/SEM 2/FYP 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="367" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E22AE2E-082F-4B3A-9366-14BFBB38D1EE}"/>
+  <xr:revisionPtr revIDLastSave="371" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{962943DE-E578-4AE5-9869-665DD3B54711}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{A67127B6-E741-4082-8256-CD80F0C0B572}"/>
   </bookViews>
@@ -17,7 +17,6 @@
     <sheet name="roadmap" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -478,26 +477,26 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1220,10 +1219,10 @@
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B5" s="21">
-        <v>1</v>
-      </c>
-      <c r="C5" s="20" t="s">
+      <c r="B5" s="23">
+        <v>1</v>
+      </c>
+      <c r="C5" s="26" t="s">
         <v>20</v>
       </c>
       <c r="D5" s="17" t="s">
@@ -1243,8 +1242,8 @@
       </c>
     </row>
     <row r="6" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B6" s="21"/>
-      <c r="C6" s="20"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="26"/>
       <c r="D6" s="17" t="s">
         <v>34</v>
       </c>
@@ -1262,10 +1261,10 @@
       </c>
     </row>
     <row r="7" spans="2:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="21">
+      <c r="B7" s="23">
         <v>2</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="23" t="s">
         <v>21</v>
       </c>
       <c r="D7" s="18" t="s">
@@ -1280,13 +1279,13 @@
       <c r="G7" s="15">
         <v>46272</v>
       </c>
-      <c r="H7" s="24" t="s">
+      <c r="H7" s="20" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B8" s="21"/>
-      <c r="C8" s="21"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
       <c r="D8" s="18" t="s">
         <v>36</v>
       </c>
@@ -1299,13 +1298,13 @@
       <c r="G8" s="15">
         <v>46272</v>
       </c>
-      <c r="H8" s="25"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B9" s="21">
+      <c r="B9" s="23">
         <v>3</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="C9" s="23" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="18" t="s">
@@ -1320,13 +1319,13 @@
       <c r="G9" s="15">
         <v>46272</v>
       </c>
-      <c r="H9" s="24" t="s">
+      <c r="H9" s="20" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B10" s="21"/>
-      <c r="C10" s="21"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="23"/>
       <c r="D10" s="18" t="s">
         <v>38</v>
       </c>
@@ -1339,13 +1338,13 @@
       <c r="G10" s="15">
         <v>46272</v>
       </c>
-      <c r="H10" s="25"/>
+      <c r="H10" s="21"/>
     </row>
     <row r="11" spans="2:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="21">
+      <c r="B11" s="23">
         <v>4</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="C11" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D11" s="18" t="s">
@@ -1360,13 +1359,13 @@
       <c r="G11" s="15">
         <v>46272</v>
       </c>
-      <c r="H11" s="24" t="s">
+      <c r="H11" s="20" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B12" s="21"/>
-      <c r="C12" s="21"/>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
       <c r="D12" s="18" t="s">
         <v>40</v>
       </c>
@@ -1379,13 +1378,13 @@
       <c r="G12" s="15">
         <v>46272</v>
       </c>
-      <c r="H12" s="25"/>
+      <c r="H12" s="21"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B13" s="21">
+      <c r="B13" s="23">
         <v>5</v>
       </c>
-      <c r="C13" s="21" t="s">
+      <c r="C13" s="23" t="s">
         <v>24</v>
       </c>
       <c r="D13" s="18" t="s">
@@ -1400,13 +1399,13 @@
       <c r="G13" s="15">
         <v>46272</v>
       </c>
-      <c r="H13" s="24" t="s">
+      <c r="H13" s="20" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B14" s="21"/>
-      <c r="C14" s="21"/>
+      <c r="B14" s="23"/>
+      <c r="C14" s="23"/>
       <c r="D14" s="18" t="s">
         <v>42</v>
       </c>
@@ -1419,11 +1418,11 @@
       <c r="G14" s="15">
         <v>46272</v>
       </c>
-      <c r="H14" s="26"/>
+      <c r="H14" s="22"/>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B15" s="21"/>
-      <c r="C15" s="21"/>
+      <c r="B15" s="23"/>
+      <c r="C15" s="23"/>
       <c r="D15" s="18" t="s">
         <v>43</v>
       </c>
@@ -1436,11 +1435,11 @@
       <c r="G15" s="15">
         <v>46272</v>
       </c>
-      <c r="H15" s="26"/>
+      <c r="H15" s="22"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B16" s="21"/>
-      <c r="C16" s="21"/>
+      <c r="B16" s="23"/>
+      <c r="C16" s="23"/>
       <c r="D16" s="18" t="s">
         <v>44</v>
       </c>
@@ -1453,11 +1452,11 @@
       <c r="G16" s="15">
         <v>46272</v>
       </c>
-      <c r="H16" s="26"/>
+      <c r="H16" s="22"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="23"/>
       <c r="D17" s="18" t="s">
         <v>45</v>
       </c>
@@ -1470,13 +1469,13 @@
       <c r="G17" s="15">
         <v>46272</v>
       </c>
-      <c r="H17" s="25"/>
+      <c r="H17" s="21"/>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B18" s="21">
+      <c r="B18" s="23">
         <v>6</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="23" t="s">
         <v>25</v>
       </c>
       <c r="D18" s="18" t="s">
@@ -1491,13 +1490,13 @@
       <c r="G18" s="15">
         <v>46272</v>
       </c>
-      <c r="H18" s="24" t="s">
+      <c r="H18" s="20" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B19" s="21"/>
-      <c r="C19" s="21"/>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
       <c r="D19" s="18" t="s">
         <v>48</v>
       </c>
@@ -1510,7 +1509,7 @@
       <c r="G19" s="15">
         <v>46272</v>
       </c>
-      <c r="H19" s="25"/>
+      <c r="H19" s="21"/>
       <c r="I19" s="1"/>
     </row>
     <row r="20" spans="2:9" ht="43.2" x14ac:dyDescent="0.3">
@@ -1538,10 +1537,10 @@
       <c r="I20" s="1"/>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B21" s="21">
+      <c r="B21" s="23">
         <v>8</v>
       </c>
-      <c r="C21" s="21" t="s">
+      <c r="C21" s="23" t="s">
         <v>10</v>
       </c>
       <c r="D21" s="18" t="s">
@@ -1556,14 +1555,14 @@
       <c r="G21" s="15">
         <v>46274</v>
       </c>
-      <c r="H21" s="24" t="s">
+      <c r="H21" s="20" t="s">
         <v>72</v>
       </c>
       <c r="I21" s="1"/>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B22" s="21"/>
-      <c r="C22" s="21"/>
+      <c r="B22" s="23"/>
+      <c r="C22" s="23"/>
       <c r="D22" s="18" t="s">
         <v>51</v>
       </c>
@@ -1576,7 +1575,7 @@
       <c r="G22" s="15">
         <v>46274</v>
       </c>
-      <c r="H22" s="25"/>
+      <c r="H22" s="21"/>
       <c r="I22" s="1"/>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.3">
@@ -1628,10 +1627,10 @@
       <c r="I24" s="1"/>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B25" s="21">
+      <c r="B25" s="23">
         <v>11</v>
       </c>
-      <c r="C25" s="21" t="s">
+      <c r="C25" s="23" t="s">
         <v>28</v>
       </c>
       <c r="D25" s="18" t="s">
@@ -1640,58 +1639,66 @@
       <c r="E25" s="14" t="b">
         <v>0</v>
       </c>
-      <c r="F25" s="15"/>
+      <c r="F25" s="15">
+        <v>46279</v>
+      </c>
       <c r="G25" s="15"/>
-      <c r="H25" s="24"/>
+      <c r="H25" s="20"/>
       <c r="I25" s="1"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B26" s="21"/>
-      <c r="C26" s="21"/>
+      <c r="B26" s="23"/>
+      <c r="C26" s="23"/>
       <c r="D26" s="18" t="s">
         <v>56</v>
       </c>
       <c r="E26" s="14" t="b">
         <v>0</v>
       </c>
-      <c r="F26" s="15"/>
+      <c r="F26" s="15">
+        <v>46279</v>
+      </c>
       <c r="G26" s="15"/>
-      <c r="H26" s="26"/>
+      <c r="H26" s="22"/>
       <c r="I26" s="1"/>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B27" s="21"/>
-      <c r="C27" s="21"/>
+      <c r="B27" s="23"/>
+      <c r="C27" s="23"/>
       <c r="D27" s="18" t="s">
         <v>57</v>
       </c>
       <c r="E27" s="14" t="b">
         <v>0</v>
       </c>
-      <c r="F27" s="15"/>
+      <c r="F27" s="15">
+        <v>46279</v>
+      </c>
       <c r="G27" s="15"/>
-      <c r="H27" s="26"/>
+      <c r="H27" s="22"/>
       <c r="I27" s="1"/>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B28" s="21"/>
-      <c r="C28" s="21"/>
+      <c r="B28" s="23"/>
+      <c r="C28" s="23"/>
       <c r="D28" s="18" t="s">
         <v>58</v>
       </c>
       <c r="E28" s="14" t="b">
         <v>0</v>
       </c>
-      <c r="F28" s="15"/>
+      <c r="F28" s="15">
+        <v>46279</v>
+      </c>
       <c r="G28" s="15"/>
-      <c r="H28" s="25"/>
+      <c r="H28" s="21"/>
       <c r="I28" s="1"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B29" s="22">
+      <c r="B29" s="24">
         <v>12</v>
       </c>
-      <c r="C29" s="21" t="s">
+      <c r="C29" s="23" t="s">
         <v>29</v>
       </c>
       <c r="D29" s="18" t="s">
@@ -1700,14 +1707,16 @@
       <c r="E29" s="14" t="b">
         <v>0</v>
       </c>
-      <c r="F29" s="15"/>
+      <c r="F29" s="15">
+        <v>46279</v>
+      </c>
       <c r="G29" s="15"/>
-      <c r="H29" s="24"/>
+      <c r="H29" s="20"/>
       <c r="I29" s="1"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B30" s="23"/>
-      <c r="C30" s="21"/>
+      <c r="B30" s="25"/>
+      <c r="C30" s="23"/>
       <c r="D30" s="18" t="s">
         <v>60</v>
       </c>
@@ -1716,7 +1725,7 @@
       </c>
       <c r="F30" s="15"/>
       <c r="G30" s="15"/>
-      <c r="H30" s="25"/>
+      <c r="H30" s="21"/>
       <c r="I30" s="1"/>
     </row>
     <row r="31" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -1755,6 +1764,24 @@
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C13:C17"/>
+    <mergeCell ref="B13:B17"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C25:C28"/>
+    <mergeCell ref="B25:B28"/>
     <mergeCell ref="H18:H19"/>
     <mergeCell ref="H21:H22"/>
     <mergeCell ref="H25:H28"/>
@@ -1763,24 +1790,6 @@
     <mergeCell ref="H9:H10"/>
     <mergeCell ref="H11:H12"/>
     <mergeCell ref="H13:H17"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C25:C28"/>
-    <mergeCell ref="B25:B28"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C13:C17"/>
-    <mergeCell ref="B13:B17"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="B9:B10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Selenium UI tests and required form fields
</commit_message>
<xml_diff>
--- a/FYP 2 Checklist.xlsx
+++ b/FYP 2 Checklist.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d63ed5ca29abe7a/Desktop/my file/UTP/SCHOOL WORK/UNDERGRADUATE/3RD YEAR/SEM 2/FYP 2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3D63ED5CA29ABE7A/Desktop/my file/UTP/SCHOOL WORK/UNDERGRADUATE/3RD YEAR/SEM 2/FYP 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="371" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{962943DE-E578-4AE5-9869-665DD3B54711}"/>
+  <xr:revisionPtr revIDLastSave="384" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA89FAE0-9949-48CF-9D1D-851F1BA4FEF1}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{A67127B6-E741-4082-8256-CD80F0C0B572}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{A67127B6-E741-4082-8256-CD80F0C0B572}"/>
   </bookViews>
   <sheets>
     <sheet name="gantt chart" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="76">
   <si>
     <t>FYP II Gantt Chart</t>
   </si>
@@ -265,6 +265,13 @@
   </si>
   <si>
     <t>auto filled right after the code is runnung</t>
+  </si>
+  <si>
+    <t>Area(Tests)
+Login and logout	(2)
+Submit bug (valid flow)	(1)
+Required-field validation	(6)
+Bug status update	(2)</t>
   </si>
 </sst>
 </file>
@@ -477,6 +484,18 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -485,18 +504,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -545,10 +552,6 @@
     </a>
   </bag>
 </FeaturePropertyBags>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1219,10 +1222,10 @@
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B5" s="23">
-        <v>1</v>
-      </c>
-      <c r="C5" s="26" t="s">
+      <c r="B5" s="21">
+        <v>1</v>
+      </c>
+      <c r="C5" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D5" s="17" t="s">
@@ -1242,8 +1245,8 @@
       </c>
     </row>
     <row r="6" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B6" s="23"/>
-      <c r="C6" s="26"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="20"/>
       <c r="D6" s="17" t="s">
         <v>34</v>
       </c>
@@ -1261,10 +1264,10 @@
       </c>
     </row>
     <row r="7" spans="2:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="23">
+      <c r="B7" s="21">
         <v>2</v>
       </c>
-      <c r="C7" s="23" t="s">
+      <c r="C7" s="21" t="s">
         <v>21</v>
       </c>
       <c r="D7" s="18" t="s">
@@ -1279,13 +1282,13 @@
       <c r="G7" s="15">
         <v>46272</v>
       </c>
-      <c r="H7" s="20" t="s">
+      <c r="H7" s="24" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B8" s="23"/>
-      <c r="C8" s="23"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="21"/>
       <c r="D8" s="18" t="s">
         <v>36</v>
       </c>
@@ -1298,13 +1301,13 @@
       <c r="G8" s="15">
         <v>46272</v>
       </c>
-      <c r="H8" s="21"/>
+      <c r="H8" s="25"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B9" s="23">
+      <c r="B9" s="21">
         <v>3</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="C9" s="21" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="18" t="s">
@@ -1319,13 +1322,13 @@
       <c r="G9" s="15">
         <v>46272</v>
       </c>
-      <c r="H9" s="20" t="s">
+      <c r="H9" s="24" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
       <c r="D10" s="18" t="s">
         <v>38</v>
       </c>
@@ -1338,13 +1341,13 @@
       <c r="G10" s="15">
         <v>46272</v>
       </c>
-      <c r="H10" s="21"/>
+      <c r="H10" s="25"/>
     </row>
     <row r="11" spans="2:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="23">
+      <c r="B11" s="21">
         <v>4</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="21" t="s">
         <v>23</v>
       </c>
       <c r="D11" s="18" t="s">
@@ -1359,13 +1362,13 @@
       <c r="G11" s="15">
         <v>46272</v>
       </c>
-      <c r="H11" s="20" t="s">
+      <c r="H11" s="24" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
       <c r="D12" s="18" t="s">
         <v>40</v>
       </c>
@@ -1378,13 +1381,13 @@
       <c r="G12" s="15">
         <v>46272</v>
       </c>
-      <c r="H12" s="21"/>
+      <c r="H12" s="25"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B13" s="23">
+      <c r="B13" s="21">
         <v>5</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="C13" s="21" t="s">
         <v>24</v>
       </c>
       <c r="D13" s="18" t="s">
@@ -1399,13 +1402,13 @@
       <c r="G13" s="15">
         <v>46272</v>
       </c>
-      <c r="H13" s="20" t="s">
+      <c r="H13" s="24" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B14" s="23"/>
-      <c r="C14" s="23"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
       <c r="D14" s="18" t="s">
         <v>42</v>
       </c>
@@ -1418,11 +1421,11 @@
       <c r="G14" s="15">
         <v>46272</v>
       </c>
-      <c r="H14" s="22"/>
+      <c r="H14" s="26"/>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B15" s="23"/>
-      <c r="C15" s="23"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
       <c r="D15" s="18" t="s">
         <v>43</v>
       </c>
@@ -1435,11 +1438,11 @@
       <c r="G15" s="15">
         <v>46272</v>
       </c>
-      <c r="H15" s="22"/>
+      <c r="H15" s="26"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
       <c r="D16" s="18" t="s">
         <v>44</v>
       </c>
@@ -1452,11 +1455,11 @@
       <c r="G16" s="15">
         <v>46272</v>
       </c>
-      <c r="H16" s="22"/>
+      <c r="H16" s="26"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
       <c r="D17" s="18" t="s">
         <v>45</v>
       </c>
@@ -1469,13 +1472,13 @@
       <c r="G17" s="15">
         <v>46272</v>
       </c>
-      <c r="H17" s="21"/>
+      <c r="H17" s="25"/>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B18" s="23">
+      <c r="B18" s="21">
         <v>6</v>
       </c>
-      <c r="C18" s="23" t="s">
+      <c r="C18" s="21" t="s">
         <v>25</v>
       </c>
       <c r="D18" s="18" t="s">
@@ -1490,13 +1493,13 @@
       <c r="G18" s="15">
         <v>46272</v>
       </c>
-      <c r="H18" s="20" t="s">
+      <c r="H18" s="24" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B19" s="23"/>
-      <c r="C19" s="23"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
       <c r="D19" s="18" t="s">
         <v>48</v>
       </c>
@@ -1509,7 +1512,7 @@
       <c r="G19" s="15">
         <v>46272</v>
       </c>
-      <c r="H19" s="21"/>
+      <c r="H19" s="25"/>
       <c r="I19" s="1"/>
     </row>
     <row r="20" spans="2:9" ht="43.2" x14ac:dyDescent="0.3">
@@ -1537,10 +1540,10 @@
       <c r="I20" s="1"/>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B21" s="23">
+      <c r="B21" s="21">
         <v>8</v>
       </c>
-      <c r="C21" s="23" t="s">
+      <c r="C21" s="21" t="s">
         <v>10</v>
       </c>
       <c r="D21" s="18" t="s">
@@ -1555,14 +1558,14 @@
       <c r="G21" s="15">
         <v>46274</v>
       </c>
-      <c r="H21" s="20" t="s">
+      <c r="H21" s="24" t="s">
         <v>72</v>
       </c>
       <c r="I21" s="1"/>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B22" s="23"/>
-      <c r="C22" s="23"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="21"/>
       <c r="D22" s="18" t="s">
         <v>51</v>
       </c>
@@ -1575,7 +1578,7 @@
       <c r="G22" s="15">
         <v>46274</v>
       </c>
-      <c r="H22" s="21"/>
+      <c r="H22" s="25"/>
       <c r="I22" s="1"/>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.3">
@@ -1627,78 +1630,88 @@
       <c r="I24" s="1"/>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B25" s="23">
+      <c r="B25" s="21">
         <v>11</v>
       </c>
-      <c r="C25" s="23" t="s">
+      <c r="C25" s="21" t="s">
         <v>28</v>
       </c>
       <c r="D25" s="18" t="s">
         <v>55</v>
       </c>
       <c r="E25" s="14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" s="15">
         <v>46279</v>
       </c>
-      <c r="G25" s="15"/>
-      <c r="H25" s="20"/>
+      <c r="G25" s="15">
+        <v>46314</v>
+      </c>
+      <c r="H25" s="24" t="s">
+        <v>75</v>
+      </c>
       <c r="I25" s="1"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B26" s="23"/>
-      <c r="C26" s="23"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
       <c r="D26" s="18" t="s">
         <v>56</v>
       </c>
       <c r="E26" s="14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F26" s="15">
         <v>46279</v>
       </c>
-      <c r="G26" s="15"/>
-      <c r="H26" s="22"/>
+      <c r="G26" s="15">
+        <v>46314</v>
+      </c>
+      <c r="H26" s="26"/>
       <c r="I26" s="1"/>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B27" s="23"/>
-      <c r="C27" s="23"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
       <c r="D27" s="18" t="s">
         <v>57</v>
       </c>
       <c r="E27" s="14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F27" s="15">
         <v>46279</v>
       </c>
-      <c r="G27" s="15"/>
-      <c r="H27" s="22"/>
+      <c r="G27" s="15">
+        <v>46314</v>
+      </c>
+      <c r="H27" s="26"/>
       <c r="I27" s="1"/>
     </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B28" s="23"/>
-      <c r="C28" s="23"/>
+    <row r="28" spans="2:9" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
       <c r="D28" s="18" t="s">
         <v>58</v>
       </c>
       <c r="E28" s="14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F28" s="15">
         <v>46279</v>
       </c>
-      <c r="G28" s="15"/>
-      <c r="H28" s="21"/>
+      <c r="G28" s="15">
+        <v>46314</v>
+      </c>
+      <c r="H28" s="25"/>
       <c r="I28" s="1"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B29" s="24">
+      <c r="B29" s="22">
         <v>12</v>
       </c>
-      <c r="C29" s="23" t="s">
+      <c r="C29" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D29" s="18" t="s">
@@ -1707,16 +1720,14 @@
       <c r="E29" s="14" t="b">
         <v>0</v>
       </c>
-      <c r="F29" s="15">
-        <v>46279</v>
-      </c>
+      <c r="F29" s="15"/>
       <c r="G29" s="15"/>
-      <c r="H29" s="20"/>
+      <c r="H29" s="24"/>
       <c r="I29" s="1"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B30" s="25"/>
-      <c r="C30" s="23"/>
+      <c r="B30" s="23"/>
+      <c r="C30" s="21"/>
       <c r="D30" s="18" t="s">
         <v>60</v>
       </c>
@@ -1725,7 +1736,7 @@
       </c>
       <c r="F30" s="15"/>
       <c r="G30" s="15"/>
-      <c r="H30" s="21"/>
+      <c r="H30" s="25"/>
       <c r="I30" s="1"/>
     </row>
     <row r="31" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -1764,24 +1775,6 @@
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C13:C17"/>
-    <mergeCell ref="B13:B17"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C25:C28"/>
-    <mergeCell ref="B25:B28"/>
     <mergeCell ref="H18:H19"/>
     <mergeCell ref="H21:H22"/>
     <mergeCell ref="H25:H28"/>
@@ -1790,6 +1783,24 @@
     <mergeCell ref="H9:H10"/>
     <mergeCell ref="H11:H12"/>
     <mergeCell ref="H13:H17"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C25:C28"/>
+    <mergeCell ref="B25:B28"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C13:C17"/>
+    <mergeCell ref="B13:B17"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="B9:B10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
modified: FYP 2 Checklist.xlsx and adding new file; IntelliBug_Usability_Test.xlsx
</commit_message>
<xml_diff>
--- a/FYP 2 Checklist.xlsx
+++ b/FYP 2 Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3D63ED5CA29ABE7A/Desktop/my file/UTP/SCHOOL WORK/UNDERGRADUATE/3RD YEAR/SEM 2/FYP 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="384" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA89FAE0-9949-48CF-9D1D-851F1BA4FEF1}"/>
+  <xr:revisionPtr revIDLastSave="386" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70AF2A3E-A51C-41DA-B980-4505F724BBA7}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{A67127B6-E741-4082-8256-CD80F0C0B572}"/>
   </bookViews>
@@ -1696,14 +1696,12 @@
         <v>58</v>
       </c>
       <c r="E28" s="14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F28" s="15">
         <v>46279</v>
       </c>
-      <c r="G28" s="15">
-        <v>46314</v>
-      </c>
+      <c r="G28" s="15"/>
       <c r="H28" s="25"/>
       <c r="I28" s="1"/>
     </row>

</xml_diff>

<commit_message>
Show each user only their own bug reports
</commit_message>
<xml_diff>
--- a/FYP 2 Checklist.xlsx
+++ b/FYP 2 Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3D63ED5CA29ABE7A/Desktop/my file/UTP/SCHOOL WORK/UNDERGRADUATE/3RD YEAR/SEM 2/FYP 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="386" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70AF2A3E-A51C-41DA-B980-4505F724BBA7}"/>
+  <xr:revisionPtr revIDLastSave="387" documentId="8_{1E43306B-5CAC-4F11-923B-A397D1D6FA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E46C0A5-CF73-4FE8-A5BB-2895DC59BF5A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{A67127B6-E741-4082-8256-CD80F0C0B572}"/>
   </bookViews>
@@ -1698,9 +1698,7 @@
       <c r="E28" s="14" t="b">
         <v>0</v>
       </c>
-      <c r="F28" s="15">
-        <v>46279</v>
-      </c>
+      <c r="F28" s="15"/>
       <c r="G28" s="15"/>
       <c r="H28" s="25"/>
       <c r="I28" s="1"/>

</xml_diff>